<commit_message>
Corrige le calcul du CA brut (mois) : dépendait de l'onglet Finances
Le CA du Tableau de bord, du Rapport Mensuel, de la Facture Propriétaire
et du graphique d'évolution mensuelle passait par une valeur intermédiaire
de l'onglet Finances, qui nécessite une ligne créée manuellement pour le
mois en cours. Sans cette ligne, le CA affichait 0 malgré des réservations
réelles ce mois-ci. Ces calculs pointent désormais directement sur
l'onglet Réservations (source de vérité), indépendamment de la saisie
mensuelle dans Finances.
</commit_message>
<xml_diff>
--- a/MG-Hote-ERP/MG_Hote_Gestion_Conciergerie.xlsx
+++ b/MG-Hote-ERP/MG_Hote_Gestion_Conciergerie.xlsx
@@ -2066,11 +2066,11 @@
     <row r="17">
       <c r="B17" s="35" t="inlineStr">
         <is>
-          <t>Revenu locatif encaissé</t>
+          <t>Revenu locatif brut</t>
         </is>
       </c>
       <c r="C17" s="41">
-        <f>SUMIFS(T_Finances[Revenu locatif],T_Finances[Bien],$C$6,T_Finances[Mois],$F$6)</f>
+        <f>SUMIFS(T_Reservations[Prix total (TTC)],T_Reservations[Bien],$C$6,T_Reservations[Mois],$F$6,T_Reservations[Statut],"&lt;&gt;Annulée")</f>
         <v/>
       </c>
     </row>
@@ -2271,11 +2271,11 @@
     <row r="8">
       <c r="B8" s="35" t="inlineStr">
         <is>
-          <t>Chiffre d'affaires total</t>
+          <t>Chiffre d'affaires brut total</t>
         </is>
       </c>
       <c r="C8" s="22">
-        <f>SUMIFS(T_Finances[Revenu locatif],T_Finances[Mois],$C$4)</f>
+        <f>SUMIFS(T_Reservations[Prix total (TTC)],T_Reservations[Mois],$C$4,T_Reservations[Statut],"&lt;&gt;Annulée")</f>
         <v/>
       </c>
     </row>
@@ -2838,11 +2838,11 @@
     <row r="11">
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>Chiffre d'affaires du mois</t>
+          <t>Chiffre d'affaires brut du mois</t>
         </is>
       </c>
       <c r="G11" s="19">
-        <f>SUMIFS(T_Finances[Revenu locatif],T_Finances[Mois],TEXT(TODAY(),"yyyy-mm"))</f>
+        <f>SUMIFS(T_Reservations[Prix total (TTC)],T_Reservations[Mois],TEXT(TODAY(),"yyyy-mm"),T_Reservations[Statut],"&lt;&gt;Annulée")</f>
         <v/>
       </c>
     </row>
@@ -3020,7 +3020,7 @@
         <v/>
       </c>
       <c r="C46" s="22">
-        <f>SUMIFS(T_Finances[Revenu locatif],T_Finances[Mois],TEXT(B46,"yyyy-mm"))</f>
+        <f>SUMIFS(T_Reservations[Prix total (TTC)],T_Reservations[Mois],TEXT(B46,"yyyy-mm"),T_Reservations[Statut],"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="D46" s="23">
@@ -3034,7 +3034,7 @@
         <v/>
       </c>
       <c r="C47" s="22">
-        <f>SUMIFS(T_Finances[Revenu locatif],T_Finances[Mois],TEXT(B47,"yyyy-mm"))</f>
+        <f>SUMIFS(T_Reservations[Prix total (TTC)],T_Reservations[Mois],TEXT(B47,"yyyy-mm"),T_Reservations[Statut],"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="D47" s="23">
@@ -3048,7 +3048,7 @@
         <v/>
       </c>
       <c r="C48" s="22">
-        <f>SUMIFS(T_Finances[Revenu locatif],T_Finances[Mois],TEXT(B48,"yyyy-mm"))</f>
+        <f>SUMIFS(T_Reservations[Prix total (TTC)],T_Reservations[Mois],TEXT(B48,"yyyy-mm"),T_Reservations[Statut],"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="D48" s="23">
@@ -3062,7 +3062,7 @@
         <v/>
       </c>
       <c r="C49" s="22">
-        <f>SUMIFS(T_Finances[Revenu locatif],T_Finances[Mois],TEXT(B49,"yyyy-mm"))</f>
+        <f>SUMIFS(T_Reservations[Prix total (TTC)],T_Reservations[Mois],TEXT(B49,"yyyy-mm"),T_Reservations[Statut],"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="D49" s="23">
@@ -3076,7 +3076,7 @@
         <v/>
       </c>
       <c r="C50" s="22">
-        <f>SUMIFS(T_Finances[Revenu locatif],T_Finances[Mois],TEXT(B50,"yyyy-mm"))</f>
+        <f>SUMIFS(T_Reservations[Prix total (TTC)],T_Reservations[Mois],TEXT(B50,"yyyy-mm"),T_Reservations[Statut],"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="D50" s="23">
@@ -3090,7 +3090,7 @@
         <v/>
       </c>
       <c r="C51" s="22">
-        <f>SUMIFS(T_Finances[Revenu locatif],T_Finances[Mois],TEXT(B51,"yyyy-mm"))</f>
+        <f>SUMIFS(T_Reservations[Prix total (TTC)],T_Reservations[Mois],TEXT(B51,"yyyy-mm"),T_Reservations[Statut],"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="D51" s="23">
@@ -3104,7 +3104,7 @@
         <v/>
       </c>
       <c r="C52" s="22">
-        <f>SUMIFS(T_Finances[Revenu locatif],T_Finances[Mois],TEXT(B52,"yyyy-mm"))</f>
+        <f>SUMIFS(T_Reservations[Prix total (TTC)],T_Reservations[Mois],TEXT(B52,"yyyy-mm"),T_Reservations[Statut],"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="D52" s="23">
@@ -3118,7 +3118,7 @@
         <v/>
       </c>
       <c r="C53" s="22">
-        <f>SUMIFS(T_Finances[Revenu locatif],T_Finances[Mois],TEXT(B53,"yyyy-mm"))</f>
+        <f>SUMIFS(T_Reservations[Prix total (TTC)],T_Reservations[Mois],TEXT(B53,"yyyy-mm"),T_Reservations[Statut],"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="D53" s="23">
@@ -3132,7 +3132,7 @@
         <v/>
       </c>
       <c r="C54" s="22">
-        <f>SUMIFS(T_Finances[Revenu locatif],T_Finances[Mois],TEXT(B54,"yyyy-mm"))</f>
+        <f>SUMIFS(T_Reservations[Prix total (TTC)],T_Reservations[Mois],TEXT(B54,"yyyy-mm"),T_Reservations[Statut],"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="D54" s="23">
@@ -3146,7 +3146,7 @@
         <v/>
       </c>
       <c r="C55" s="22">
-        <f>SUMIFS(T_Finances[Revenu locatif],T_Finances[Mois],TEXT(B55,"yyyy-mm"))</f>
+        <f>SUMIFS(T_Reservations[Prix total (TTC)],T_Reservations[Mois],TEXT(B55,"yyyy-mm"),T_Reservations[Statut],"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="D55" s="23">
@@ -3160,7 +3160,7 @@
         <v/>
       </c>
       <c r="C56" s="22">
-        <f>SUMIFS(T_Finances[Revenu locatif],T_Finances[Mois],TEXT(B56,"yyyy-mm"))</f>
+        <f>SUMIFS(T_Reservations[Prix total (TTC)],T_Reservations[Mois],TEXT(B56,"yyyy-mm"),T_Reservations[Statut],"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="D56" s="23">
@@ -3174,7 +3174,7 @@
         <v/>
       </c>
       <c r="C57" s="22">
-        <f>SUMIFS(T_Finances[Revenu locatif],T_Finances[Mois],TEXT(B57,"yyyy-mm"))</f>
+        <f>SUMIFS(T_Reservations[Prix total (TTC)],T_Reservations[Mois],TEXT(B57,"yyyy-mm"),T_Reservations[Statut],"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="D57" s="23">

</xml_diff>